<commit_message>
atualiza volumes loa com ppo - 22092026
</commit_message>
<xml_diff>
--- a/bancos/manual/desc_classificacao_economica_despesa.xlsx
+++ b/bancos/manual/desc_classificacao_economica_despesa.xlsx
@@ -1,26 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29301"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m753205\Desktop\99 TABELAS APOIO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\x1569275\CAMG\Splor Geral - @dcppn\00- DCPPN 2027\PPAG e LOA 2027\Dados para Volumes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_720F13E4720CF0ED19868A9C9DEB84F5CECEC513" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A657D371-65EE-4C3C-9D92-636BB04CCE07}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21600" windowHeight="8400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21600" windowHeight="8400"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Plan1!$A$1:$B$219</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Plan1!$A$1:$B$221</definedName>
     <definedName name="_GoBack" localSheetId="0">Plan1!#REF!</definedName>
     <definedName name="LOCAL_MYSQL_DATE_FORMAT" hidden="1">REPT(LOCAL_YEAR_FORMAT,4)&amp;LOCAL_DATE_SEPARATOR&amp;REPT(LOCAL_MONTH_FORMAT,2)&amp;LOCAL_DATE_SEPARATOR&amp;REPT(LOCAL_DAY_FORMAT,2)&amp;" "&amp;REPT(LOCAL_HOUR_FORMAT,2)&amp;LOCAL_TIME_SEPARATOR&amp;REPT(LOCAL_MINUTE_FORMAT,2)&amp;LOCAL_TIME_SEPARATOR&amp;REPT(LOCAL_SECOND_FORMAT,2)</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="330">
   <si>
     <t>codigo</t>
   </si>
@@ -1025,13 +1024,19 @@
   </si>
   <si>
     <t>RESERVA DE CONTINGÊNCIA</t>
+  </si>
+  <si>
+    <t>4 5 90 84</t>
+  </si>
+  <si>
+    <t>4 4 46 42</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1360,15 +1365,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B219"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B221"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.85546875" style="1" customWidth="1"/>
     <col min="2" max="2" width="76.5703125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1376,7 +1381,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -1384,7 +1389,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1392,7 +1397,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1400,7 +1405,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -1408,7 +1413,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -1416,7 +1421,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -1424,7 +1429,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -1432,7 +1437,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -1440,7 +1445,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
@@ -1448,7 +1453,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -1456,7 +1461,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
@@ -1464,7 +1469,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>24</v>
       </c>
@@ -1472,7 +1477,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
@@ -1480,7 +1485,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
@@ -1488,7 +1493,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
@@ -1496,7 +1501,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
@@ -1504,7 +1509,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
@@ -1512,7 +1517,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>36</v>
       </c>
@@ -1520,7 +1525,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>38</v>
       </c>
@@ -1528,7 +1533,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>40</v>
       </c>
@@ -1536,7 +1541,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>42</v>
       </c>
@@ -1544,7 +1549,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>44</v>
       </c>
@@ -1552,7 +1557,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>45</v>
       </c>
@@ -1560,7 +1565,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>46</v>
       </c>
@@ -1568,7 +1573,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>47</v>
       </c>
@@ -1576,7 +1581,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>48</v>
       </c>
@@ -1584,7 +1589,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="1:2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>50</v>
       </c>
@@ -1592,7 +1597,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="29" spans="1:2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>52</v>
       </c>
@@ -1600,7 +1605,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="30" spans="1:2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>54</v>
       </c>
@@ -1608,7 +1613,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="31" spans="1:2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>56</v>
       </c>
@@ -1616,7 +1621,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="32" spans="1:2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>58</v>
       </c>
@@ -1624,7 +1629,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>60</v>
       </c>
@@ -1632,7 +1637,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="34" spans="1:2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>62</v>
       </c>
@@ -1640,7 +1645,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>63</v>
       </c>
@@ -1648,7 +1653,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="36" spans="1:2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>64</v>
       </c>
@@ -1656,7 +1661,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="37" spans="1:2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>65</v>
       </c>
@@ -1664,7 +1669,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="38" spans="1:2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>67</v>
       </c>
@@ -1672,7 +1677,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="39" spans="1:2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>69</v>
       </c>
@@ -1680,7 +1685,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="40" spans="1:2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>71</v>
       </c>
@@ -1688,7 +1693,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="41" spans="1:2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>72</v>
       </c>
@@ -1696,7 +1701,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="42" spans="1:2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>73</v>
       </c>
@@ -1704,7 +1709,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="43" spans="1:2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>74</v>
       </c>
@@ -1712,7 +1717,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="44" spans="1:2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>76</v>
       </c>
@@ -1720,7 +1725,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="45" spans="1:2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>77</v>
       </c>
@@ -1728,7 +1733,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="46" spans="1:2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>78</v>
       </c>
@@ -1736,7 +1741,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="47" spans="1:2">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>80</v>
       </c>
@@ -1744,7 +1749,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="48" spans="1:2">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>82</v>
       </c>
@@ -1752,7 +1757,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="49" spans="1:2">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>83</v>
       </c>
@@ -1760,7 +1765,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="50" spans="1:2">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>85</v>
       </c>
@@ -1768,7 +1773,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="51" spans="1:2">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>87</v>
       </c>
@@ -1776,7 +1781,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="52" spans="1:2">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>89</v>
       </c>
@@ -1784,7 +1789,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="53" spans="1:2">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>90</v>
       </c>
@@ -1792,7 +1797,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="54" spans="1:2">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>91</v>
       </c>
@@ -1800,7 +1805,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="55" spans="1:2">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>93</v>
       </c>
@@ -1808,7 +1813,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="56" spans="1:2">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>95</v>
       </c>
@@ -1816,7 +1821,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="57" spans="1:2">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>96</v>
       </c>
@@ -1824,7 +1829,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="58" spans="1:2">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>97</v>
       </c>
@@ -1832,7 +1837,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="59" spans="1:2">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>99</v>
       </c>
@@ -1840,7 +1845,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="60" spans="1:2">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>100</v>
       </c>
@@ -1848,7 +1853,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="61" spans="1:2">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>102</v>
       </c>
@@ -1856,7 +1861,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="62" spans="1:2">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>103</v>
       </c>
@@ -1864,7 +1869,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="63" spans="1:2">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>105</v>
       </c>
@@ -1872,7 +1877,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="64" spans="1:2">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>107</v>
       </c>
@@ -1880,7 +1885,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="65" spans="1:2">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>109</v>
       </c>
@@ -1888,7 +1893,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="66" spans="1:2">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>111</v>
       </c>
@@ -1896,7 +1901,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="67" spans="1:2">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>112</v>
       </c>
@@ -1904,7 +1909,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="68" spans="1:2">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>114</v>
       </c>
@@ -1912,7 +1917,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="69" spans="1:2">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>115</v>
       </c>
@@ -1920,7 +1925,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="70" spans="1:2">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>116</v>
       </c>
@@ -1928,7 +1933,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="71" spans="1:2">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>118</v>
       </c>
@@ -1936,7 +1941,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="72" spans="1:2">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>120</v>
       </c>
@@ -1944,7 +1949,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="73" spans="1:2">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>121</v>
       </c>
@@ -1952,7 +1957,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="74" spans="1:2">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>123</v>
       </c>
@@ -1960,7 +1965,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="75" spans="1:2">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>124</v>
       </c>
@@ -1968,7 +1973,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="76" spans="1:2">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>125</v>
       </c>
@@ -1976,7 +1981,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="77" spans="1:2">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>127</v>
       </c>
@@ -1984,7 +1989,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="78" spans="1:2">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>129</v>
       </c>
@@ -1992,7 +1997,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="79" spans="1:2">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>130</v>
       </c>
@@ -2000,7 +2005,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="80" spans="1:2">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>132</v>
       </c>
@@ -2008,7 +2013,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="81" spans="1:2">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>134</v>
       </c>
@@ -2016,7 +2021,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="82" spans="1:2">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>136</v>
       </c>
@@ -2024,7 +2029,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="83" spans="1:2">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>138</v>
       </c>
@@ -2032,7 +2037,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="84" spans="1:2">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>140</v>
       </c>
@@ -2040,7 +2045,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="85" spans="1:2">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>142</v>
       </c>
@@ -2048,7 +2053,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="86" spans="1:2">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>144</v>
       </c>
@@ -2056,7 +2061,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="87" spans="1:2">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>146</v>
       </c>
@@ -2064,7 +2069,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="88" spans="1:2">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>148</v>
       </c>
@@ -2072,7 +2077,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="89" spans="1:2">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>150</v>
       </c>
@@ -2080,7 +2085,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="90" spans="1:2">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>152</v>
       </c>
@@ -2088,7 +2093,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="91" spans="1:2">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>153</v>
       </c>
@@ -2096,7 +2101,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="92" spans="1:2">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>155</v>
       </c>
@@ -2104,7 +2109,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="93" spans="1:2">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>157</v>
       </c>
@@ -2112,7 +2117,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="94" spans="1:2">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>159</v>
       </c>
@@ -2120,7 +2125,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="95" spans="1:2">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>161</v>
       </c>
@@ -2128,7 +2133,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="96" spans="1:2">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>163</v>
       </c>
@@ -2136,7 +2141,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="97" spans="1:2">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>164</v>
       </c>
@@ -2144,7 +2149,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="98" spans="1:2">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>166</v>
       </c>
@@ -2152,7 +2157,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="99" spans="1:2">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>168</v>
       </c>
@@ -2160,7 +2165,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="100" spans="1:2">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>169</v>
       </c>
@@ -2168,7 +2173,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="101" spans="1:2">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>171</v>
       </c>
@@ -2176,7 +2181,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="102" spans="1:2">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>172</v>
       </c>
@@ -2184,7 +2189,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="103" spans="1:2">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>174</v>
       </c>
@@ -2192,7 +2197,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="104" spans="1:2">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>176</v>
       </c>
@@ -2200,7 +2205,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="105" spans="1:2">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>178</v>
       </c>
@@ -2208,7 +2213,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="106" spans="1:2">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>180</v>
       </c>
@@ -2216,7 +2221,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="107" spans="1:2">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>182</v>
       </c>
@@ -2224,7 +2229,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="108" spans="1:2">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>183</v>
       </c>
@@ -2232,7 +2237,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="109" spans="1:2">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>184</v>
       </c>
@@ -2240,7 +2245,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="110" spans="1:2">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
         <v>186</v>
       </c>
@@ -2248,7 +2253,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="111" spans="1:2">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>188</v>
       </c>
@@ -2256,7 +2261,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="112" spans="1:2">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>190</v>
       </c>
@@ -2264,7 +2269,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="113" spans="1:2">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>191</v>
       </c>
@@ -2272,7 +2277,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="114" spans="1:2">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
         <v>192</v>
       </c>
@@ -2280,7 +2285,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="115" spans="1:2">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>193</v>
       </c>
@@ -2288,7 +2293,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="116" spans="1:2">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
         <v>195</v>
       </c>
@@ -2296,7 +2301,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="117" spans="1:2">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>197</v>
       </c>
@@ -2304,7 +2309,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="118" spans="1:2">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
         <v>199</v>
       </c>
@@ -2312,7 +2317,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="119" spans="1:2">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>200</v>
       </c>
@@ -2320,7 +2325,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="120" spans="1:2">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
         <v>201</v>
       </c>
@@ -2328,7 +2333,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="121" spans="1:2">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
         <v>202</v>
       </c>
@@ -2336,7 +2341,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="122" spans="1:2">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
         <v>203</v>
       </c>
@@ -2344,7 +2349,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="123" spans="1:2">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>204</v>
       </c>
@@ -2352,7 +2357,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="124" spans="1:2">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
         <v>205</v>
       </c>
@@ -2360,7 +2365,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="125" spans="1:2">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
         <v>206</v>
       </c>
@@ -2368,7 +2373,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="126" spans="1:2">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
         <v>207</v>
       </c>
@@ -2376,7 +2381,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="127" spans="1:2">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
         <v>208</v>
       </c>
@@ -2384,7 +2389,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="128" spans="1:2">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
         <v>209</v>
       </c>
@@ -2392,7 +2397,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="129" spans="1:2">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
         <v>210</v>
       </c>
@@ -2400,7 +2405,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="130" spans="1:2">
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
         <v>212</v>
       </c>
@@ -2408,7 +2413,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="131" spans="1:2">
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
         <v>213</v>
       </c>
@@ -2416,7 +2421,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="132" spans="1:2">
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
         <v>214</v>
       </c>
@@ -2424,7 +2429,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="133" spans="1:2">
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
         <v>215</v>
       </c>
@@ -2432,7 +2437,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="134" spans="1:2">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
         <v>216</v>
       </c>
@@ -2440,7 +2445,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="135" spans="1:2">
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
         <v>217</v>
       </c>
@@ -2448,7 +2453,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="136" spans="1:2">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
         <v>218</v>
       </c>
@@ -2456,7 +2461,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="137" spans="1:2">
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
         <v>219</v>
       </c>
@@ -2464,7 +2469,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="138" spans="1:2">
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A138" s="1" t="s">
         <v>221</v>
       </c>
@@ -2472,7 +2477,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="139" spans="1:2">
+    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A139" s="1" t="s">
         <v>223</v>
       </c>
@@ -2480,7 +2485,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="140" spans="1:2">
+    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
         <v>224</v>
       </c>
@@ -2488,7 +2493,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="141" spans="1:2">
+    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
         <v>225</v>
       </c>
@@ -2496,7 +2501,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="142" spans="1:2">
+    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
         <v>226</v>
       </c>
@@ -2504,7 +2509,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="143" spans="1:2">
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
         <v>227</v>
       </c>
@@ -2512,7 +2517,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="144" spans="1:2">
+    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
         <v>228</v>
       </c>
@@ -2520,7 +2525,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="145" spans="1:2">
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
         <v>230</v>
       </c>
@@ -2528,7 +2533,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="146" spans="1:2">
+    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
         <v>232</v>
       </c>
@@ -2536,592 +2541,608 @@
         <v>70</v>
       </c>
     </row>
-    <row r="147" spans="1:2">
+    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="B147" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A148" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="B147" s="1" t="s">
+      <c r="B148" s="1" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="148" spans="1:2">
-      <c r="A148" s="1" t="s">
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A149" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="B148" s="1" t="s">
+      <c r="B149" s="1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="149" spans="1:2">
-      <c r="A149" s="1" t="s">
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A150" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="B149" s="1" t="s">
+      <c r="B150" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="150" spans="1:2">
-      <c r="A150" s="1" t="s">
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A151" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="B150" s="1" t="s">
+      <c r="B151" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="151" spans="1:2">
-      <c r="A151" s="1" t="s">
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A152" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="B151" s="1" t="s">
+      <c r="B152" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="152" spans="1:2">
-      <c r="A152" s="1" t="s">
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A153" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="B152" s="1" t="s">
+      <c r="B153" s="1" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="153" spans="1:2">
-      <c r="A153" s="1" t="s">
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A154" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="B153" s="1" t="s">
+      <c r="B154" s="1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="154" spans="1:2">
-      <c r="A154" s="1" t="s">
+    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A155" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="B154" s="1" t="s">
+      <c r="B155" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="155" spans="1:2">
-      <c r="A155" s="1" t="s">
+    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A156" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="B155" s="1" t="s">
+      <c r="B156" s="1" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="156" spans="1:2">
-      <c r="A156" s="1" t="s">
+    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A157" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="B156" s="1" t="s">
+      <c r="B157" s="1" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="157" spans="1:2">
-      <c r="A157" s="1" t="s">
+    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A158" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="B157" s="1" t="s">
+      <c r="B158" s="1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="158" spans="1:2">
-      <c r="A158" s="1" t="s">
+    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A159" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="B158" s="1" t="s">
+      <c r="B159" s="1" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="159" spans="1:2">
-      <c r="A159" s="1" t="s">
+    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A160" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="B159" s="2" t="s">
+      <c r="B160" s="2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="160" spans="1:2">
-      <c r="A160" s="1" t="s">
+    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A161" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="B160" s="1" t="s">
+      <c r="B161" s="1" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="161" spans="1:2">
-      <c r="A161" s="1" t="s">
+    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A162" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="B161" s="1" t="s">
+      <c r="B162" s="1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="162" spans="1:2">
-      <c r="A162" s="1" t="s">
+    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A163" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="B162" s="1" t="s">
+      <c r="B163" s="1" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="163" spans="1:2">
-      <c r="A163" s="1" t="s">
+    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A164" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="B163" s="1" t="s">
+      <c r="B164" s="1" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="164" spans="1:2">
-      <c r="A164" s="1" t="s">
+    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A165" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="B164" s="1" t="s">
+      <c r="B165" s="1" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="165" spans="1:2">
-      <c r="A165" s="1" t="s">
+    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A166" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="B165" s="1" t="s">
+      <c r="B166" s="1" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="166" spans="1:2">
-      <c r="A166" s="1" t="s">
+    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A167" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="B166" s="1" t="s">
+      <c r="B167" s="1" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="167" spans="1:2">
-      <c r="A167" s="1" t="s">
+    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A168" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="B167" s="1" t="s">
+      <c r="B168" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="168" spans="1:2">
-      <c r="A168" s="1" t="s">
+    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A169" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="B168" s="1" t="s">
+      <c r="B169" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="169" spans="1:2">
-      <c r="A169" s="1" t="s">
+    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A170" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="B169" s="1" t="s">
+      <c r="B170" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="170" spans="1:2">
-      <c r="A170" s="1" t="s">
+    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A171" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="B170" s="1" t="s">
+      <c r="B171" s="1" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="171" spans="1:2">
-      <c r="A171" s="1" t="s">
+    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A172" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="B171" s="1" t="s">
+      <c r="B172" s="1" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="172" spans="1:2">
-      <c r="A172" s="1" t="s">
+    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A173" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="B172" s="1" t="s">
+      <c r="B173" s="1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="173" spans="1:2">
-      <c r="A173" s="1" t="s">
+    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A174" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="B173" s="1" t="s">
+      <c r="B174" s="1" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="174" spans="1:2">
-      <c r="A174" s="1" t="s">
+    <row r="175" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A175" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="B174" s="1" t="s">
+      <c r="B175" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="175" spans="1:2">
-      <c r="A175" s="1" t="s">
+    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A176" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="B175" s="1" t="s">
+      <c r="B176" s="1" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="176" spans="1:2">
-      <c r="A176" s="1" t="s">
+    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A177" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="B176" s="2" t="s">
+      <c r="B177" s="2" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="177" spans="1:2">
-      <c r="A177" s="1" t="s">
+    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A178" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="B177" s="1" t="s">
+      <c r="B178" s="1" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="178" spans="1:2">
-      <c r="A178" s="1" t="s">
+    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A179" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="B178" s="2" t="s">
+      <c r="B179" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="179" spans="1:2">
-      <c r="A179" s="1" t="s">
+    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A180" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="B179" s="1" t="s">
+      <c r="B180" s="1" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="180" spans="1:2">
-      <c r="A180" s="1" t="s">
+    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A181" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="B180" s="1" t="s">
+      <c r="B181" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="181" spans="1:2">
-      <c r="A181" s="1" t="s">
+    <row r="182" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A182" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="B181" s="1" t="s">
+      <c r="B182" s="1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="182" spans="1:2">
-      <c r="A182" s="1" t="s">
+    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A183" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="B182" s="1" t="s">
+      <c r="B183" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="183" spans="1:2">
-      <c r="A183" s="1" t="s">
+    <row r="184" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A184" s="1" t="s">
         <v>276</v>
-      </c>
-      <c r="B183" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="184" spans="1:2">
-      <c r="A184" s="1" t="s">
-        <v>277</v>
       </c>
       <c r="B184" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="185" spans="1:2">
+    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A185" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B185" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="186" spans="1:2">
+    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A186" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="B186" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A187" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="B186" s="1" t="s">
+      <c r="B187" s="1" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="187" spans="1:2">
-      <c r="A187" s="1" t="s">
+    <row r="188" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A188" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="B187" s="1" t="s">
+      <c r="B188" s="1" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="188" spans="1:2">
-      <c r="A188" s="1" t="s">
+    <row r="189" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A189" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="B188" s="1" t="s">
+      <c r="B189" s="1" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="189" spans="1:2">
-      <c r="A189" s="1" t="s">
+    <row r="190" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A190" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="B189" s="1" t="s">
+      <c r="B190" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="190" spans="1:2">
-      <c r="A190" s="1" t="s">
+    <row r="191" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A191" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="B190" s="1" t="s">
+      <c r="B191" s="1" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="191" spans="1:2">
-      <c r="A191" s="1" t="s">
+    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A192" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="B191" s="1" t="s">
+      <c r="B192" s="1" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="192" spans="1:2">
-      <c r="A192" s="1" t="s">
+    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A193" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="B192" s="1" t="s">
+      <c r="B193" s="1" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="193" spans="1:2">
-      <c r="A193" s="1" t="s">
+    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A194" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="B193" s="1" t="s">
+      <c r="B194" s="1" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="194" spans="1:2">
-      <c r="A194" s="1" t="s">
+    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A195" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="B194" s="1" t="s">
+      <c r="B195" s="1" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="195" spans="1:2">
-      <c r="A195" s="1" t="s">
+    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A196" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="B195" s="1" t="s">
+      <c r="B196" s="1" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="196" spans="1:2">
-      <c r="A196" s="1" t="s">
+    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A197" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="B196" s="1" t="s">
+      <c r="B197" s="1" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="197" spans="1:2">
-      <c r="A197" s="1" t="s">
+    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A198" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="B197" s="1" t="s">
+      <c r="B198" s="1" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="198" spans="1:2">
-      <c r="A198" s="1" t="s">
+    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A199" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="B198" s="1" t="s">
+      <c r="B199" s="1" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="199" spans="1:2">
-      <c r="A199" s="1" t="s">
+    <row r="200" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A200" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="B199" s="1" t="s">
+      <c r="B200" s="1" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="200" spans="1:2">
-      <c r="A200" s="1" t="s">
+    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A201" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="B200" s="1" t="s">
+      <c r="B201" s="1" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="201" spans="1:2">
-      <c r="A201" s="1" t="s">
+    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A202" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="B201" s="1" t="s">
+      <c r="B202" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="202" spans="1:2">
-      <c r="A202" s="1" t="s">
+    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A203" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="B203" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A204" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="B202" s="1" t="s">
+      <c r="B204" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="203" spans="1:2">
-      <c r="A203" s="1" t="s">
+    <row r="205" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A205" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="B203" s="1" t="s">
+      <c r="B205" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="204" spans="1:2">
-      <c r="A204" s="1" t="s">
+    <row r="206" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A206" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="B204" s="1" t="s">
+      <c r="B206" s="1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="205" spans="1:2">
-      <c r="A205" s="1" t="s">
+    <row r="207" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A207" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="B205" s="1" t="s">
+      <c r="B207" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="206" spans="1:2">
-      <c r="A206" s="1" t="s">
+    <row r="208" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A208" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="B206" s="1" t="s">
+      <c r="B208" s="1" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="207" spans="1:2">
-      <c r="A207" s="1" t="s">
+    <row r="209" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A209" s="1" t="s">
         <v>307</v>
       </c>
-      <c r="B207" s="1" t="s">
+      <c r="B209" s="1" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="208" spans="1:2">
-      <c r="A208" s="1" t="s">
+    <row r="210" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A210" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="B208" s="1" t="s">
+      <c r="B210" s="1" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="209" spans="1:2">
-      <c r="A209" s="1" t="s">
+    <row r="211" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A211" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="B209" s="1" t="s">
+      <c r="B211" s="1" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="210" spans="1:2">
-      <c r="A210" s="1" t="s">
+    <row r="212" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A212" s="1" t="s">
         <v>313</v>
       </c>
-      <c r="B210" s="2" t="s">
+      <c r="B212" s="2" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="211" spans="1:2">
-      <c r="A211" s="1" t="s">
+    <row r="213" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A213" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="B211" s="2" t="s">
+      <c r="B213" s="2" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="212" spans="1:2">
-      <c r="A212" s="1" t="s">
+    <row r="214" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A214" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="B212" s="2" t="s">
+      <c r="B214" s="2" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="213" spans="1:2">
-      <c r="A213" s="1" t="s">
+    <row r="215" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A215" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="B213" s="2" t="s">
+      <c r="B215" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="214" spans="1:2">
-      <c r="A214" s="1" t="s">
+    <row r="216" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A216" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="B214" s="2" t="s">
+      <c r="B216" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="215" spans="1:2">
-      <c r="A215" s="1" t="s">
+    <row r="217" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A217" s="1" t="s">
         <v>321</v>
-      </c>
-      <c r="B215" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="216" spans="1:2">
-      <c r="A216" s="1" t="s">
-        <v>322</v>
-      </c>
-      <c r="B216" s="2" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="217" spans="1:2">
-      <c r="A217" s="1" t="s">
-        <v>323</v>
       </c>
       <c r="B217" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="218" spans="1:2">
+    <row r="218" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A218" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="B218" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A219" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="B219" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A220" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="B218" s="2" t="s">
+      <c r="B220" s="2" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="219" spans="1:2">
-      <c r="A219" s="1" t="s">
+    <row r="221" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A221" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="B219" s="2" t="s">
+      <c r="B221" s="2" t="s">
         <v>327</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B211">
+  <sortState ref="A2:B211">
     <sortCondition ref="A2:A211"/>
   </sortState>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -3148,15 +3169,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B08D58FADB61F04EBBB4F355C06EFBED" ma:contentTypeVersion="19" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="b1e0f6055e0e9a4b9e75d6c71ee7de91">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6f4338ef-addb-4c87-aefe-1895241b335f" xmlns:ns3="b91e7f20-fe0a-487d-91a9-605ac1c64acf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b43930f3490e4d4da1ab3f8da7df6f51" ns2:_="" ns3:_="">
     <xsd:import namespace="6f4338ef-addb-4c87-aefe-1895241b335f"/>
@@ -3417,14 +3429,55 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3A2F31B-1B5F-4D6E-B2EC-ACD111D3DDB3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3A2F31B-1B5F-4D6E-B2EC-ACD111D3DDB3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{902F26F7-5B6F-45AE-8405-7115E4FB3B39}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D10EAF9C-DA32-40C6-855D-B6EAE8C97B6E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
+    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D10EAF9C-DA32-40C6-855D-B6EAE8C97B6E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{902F26F7-5B6F-45AE-8405-7115E4FB3B39}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>